<commit_message>
Matriz de cambios SC-12 a SC-17, Product Backlog y Epicas con las 24 historias, Vision 1.1 y mailmap
</commit_message>
<xml_diff>
--- a/FASE 2/Evidencias Proyecto/Evidencias de documentación/Control del proyecto/Matriz_Control_de_Cambio_FitSearch.xlsx
+++ b/FASE 2/Evidencias Proyecto/Evidencias de documentación/Control del proyecto/Matriz_Control_de_Cambio_FitSearch.xlsx
@@ -737,7 +737,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1513,43 +1513,403 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="16" t="n"/>
-      <c r="B14" s="17" t="n"/>
-      <c r="C14" s="17" t="n"/>
-      <c r="D14" s="17" t="n"/>
-      <c r="E14" s="17" t="n"/>
-      <c r="F14" s="17" t="n"/>
-      <c r="G14" s="17" t="n"/>
-      <c r="H14" s="17" t="n"/>
-      <c r="I14" s="17" t="n"/>
-      <c r="J14" s="17" t="n"/>
-      <c r="K14" s="17" t="n"/>
-      <c r="L14" s="18" t="n"/>
-    </row>
-    <row r="16" ht="15" customHeight="1">
-      <c r="A16" s="28" t="inlineStr">
+    <row r="14" ht="113" customHeight="1">
+      <c r="A14" s="23" t="inlineStr">
+        <is>
+          <t>SC-12</t>
+        </is>
+      </c>
+      <c r="B14" s="24" t="inlineStr">
+        <is>
+          <t>Rodrigo Cárcamo Rojas / Product Owner</t>
+        </is>
+      </c>
+      <c r="C14" s="25" t="inlineStr">
+        <is>
+          <t>04-10-2026</t>
+        </is>
+      </c>
+      <c r="D14" s="25" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+      <c r="E14" s="25" t="inlineStr">
+        <is>
+          <t>Necesario</t>
+        </is>
+      </c>
+      <c r="F14" s="25" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="G14" s="24" t="inlineStr">
+        <is>
+          <t>Definir el flujo del profesional según el mockup del Product Owner: al elegir la cuenta profesional no completa datos personales, objetivos ni salud; completa su ficha profesional y entra a un espacio propio con Inicio (saludo, tareas, accesos rápidos y resumen semanal), Agenda, Perfil profesional con pestañas y las secciones Clientes, Mensajes, Reportes y Configuración como «Próximamente». Se implementó en los PR #12 y #13.</t>
+        </is>
+      </c>
+      <c r="H14" s="25" t="inlineStr">
+        <is>
+          <t>FS-HU-02, FS-HU-04</t>
+        </is>
+      </c>
+      <c r="I14" s="25" t="inlineStr">
+        <is>
+          <t>CU-02, CU-04</t>
+        </is>
+      </c>
+      <c r="J14" s="24" t="inlineStr">
+        <is>
+          <t>Fase 2 – Sprint 3 (semanas 9 y 10)</t>
+        </is>
+      </c>
+      <c r="K14" s="25" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="L14" s="26" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="83" customHeight="1">
+      <c r="A15" s="23" t="inlineStr">
+        <is>
+          <t>SC-13</t>
+        </is>
+      </c>
+      <c r="B15" s="24" t="inlineStr">
+        <is>
+          <t>Rodrigo Cárcamo Rojas / Product Owner</t>
+        </is>
+      </c>
+      <c r="C15" s="25" t="inlineStr">
+        <is>
+          <t>05-10-2026</t>
+        </is>
+      </c>
+      <c r="D15" s="25" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+      <c r="E15" s="25" t="inlineStr">
+        <is>
+          <t>Necesario</t>
+        </is>
+      </c>
+      <c r="F15" s="25" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+      <c r="G15" s="24" t="inlineStr">
+        <is>
+          <t>Mostrar el clima en el Inicio del profesional: el backend consulta Open-Meteo con las coordenadas de la ficha (redondeadas), guarda la respuesta 30 minutos y, si no hay ficha, usa Santiago. Endpoint GET /api/clima solo para profesionales (decisión D26 del DAS).</t>
+        </is>
+      </c>
+      <c r="H15" s="25" t="inlineStr">
+        <is>
+          <t>FS-HU-04</t>
+        </is>
+      </c>
+      <c r="I15" s="25" t="inlineStr">
+        <is>
+          <t>CU-04</t>
+        </is>
+      </c>
+      <c r="J15" s="24" t="inlineStr">
+        <is>
+          <t>Fase 2 – Sprint 3 (semanas 9 y 10)</t>
+        </is>
+      </c>
+      <c r="K15" s="25" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+      <c r="L15" s="26" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="113" customHeight="1">
+      <c r="A16" s="23" t="inlineStr">
+        <is>
+          <t>SC-14</t>
+        </is>
+      </c>
+      <c r="B16" s="24" t="inlineStr">
+        <is>
+          <t>Rodrigo Cárcamo Rojas / Product Owner</t>
+        </is>
+      </c>
+      <c r="C16" s="25" t="inlineStr">
+        <is>
+          <t>05-10-2026</t>
+        </is>
+      </c>
+      <c r="D16" s="25" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+      <c r="E16" s="25" t="inlineStr">
+        <is>
+          <t>Necesario</t>
+        </is>
+      </c>
+      <c r="F16" s="25" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="G16" s="24" t="inlineStr">
+        <is>
+          <t>Ajustar el menú del usuario según el mockup del Asistente de IA: «Historial de chats» sale del menú lateral y pasará a estar dentro del Asistente (FS-HU-07); se agrega «Comidas» como «Próximamente» (FS-HU-09 y FS-HU-10, macronutrientes solo de lo consumido) y se quitan las farmacias del menú, los accesos rápidos, la portada y el Inicio (quedan centros de salud y gimnasios).</t>
+        </is>
+      </c>
+      <c r="H16" s="25" t="inlineStr">
+        <is>
+          <t>FS-HU-07, FS-HU-10, FS-HU-20, FS-HU-21</t>
+        </is>
+      </c>
+      <c r="I16" s="25" t="inlineStr">
+        <is>
+          <t>CU-01, CU-05, CU-06</t>
+        </is>
+      </c>
+      <c r="J16" s="24" t="inlineStr">
+        <is>
+          <t>Fase 2 – Sprint 3 (semanas 9 y 10)</t>
+        </is>
+      </c>
+      <c r="K16" s="25" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="L16" s="26" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="113" customHeight="1">
+      <c r="A17" s="23" t="inlineStr">
+        <is>
+          <t>SC-15</t>
+        </is>
+      </c>
+      <c r="B17" s="24" t="inlineStr">
+        <is>
+          <t>Rodrigo Cárcamo Rojas / Product Owner</t>
+        </is>
+      </c>
+      <c r="C17" s="25" t="inlineStr">
+        <is>
+          <t>08-10-2026</t>
+        </is>
+      </c>
+      <c r="D17" s="25" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="E17" s="25" t="inlineStr">
+        <is>
+          <t>Urgente</t>
+        </is>
+      </c>
+      <c r="F17" s="25" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="G17" s="24" t="inlineStr">
+        <is>
+          <t>Corregir el cambio SC-08: el tipo de cuenta se elige una sola vez en una pantalla propia (/elegir-perfil) después del registro o del ingreso con Google, y no en el paso 1 del asistente, que vuelve a tener 4 pasos. Cambiarlo después lo hace un administrador (409 si ya se eligió). El profesional no accede a las pantallas ni a la API del usuario (decisión D25 del DAS, que reemplaza a D21).</t>
+        </is>
+      </c>
+      <c r="H17" s="25" t="inlineStr">
+        <is>
+          <t>FS-HU-02, FS-HU-16, FS-HU-17</t>
+        </is>
+      </c>
+      <c r="I17" s="25" t="inlineStr">
+        <is>
+          <t>CU-01, CU-02</t>
+        </is>
+      </c>
+      <c r="J17" s="24" t="inlineStr">
+        <is>
+          <t>Fase 2 – Sprint 3 (semanas 9 y 10)</t>
+        </is>
+      </c>
+      <c r="K17" s="25" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="L17" s="26" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="113" customHeight="1">
+      <c r="A18" s="23" t="inlineStr">
+        <is>
+          <t>SC-16</t>
+        </is>
+      </c>
+      <c r="B18" s="24" t="inlineStr">
+        <is>
+          <t>Rodrigo Cárcamo Rojas / Product Owner</t>
+        </is>
+      </c>
+      <c r="C18" s="25" t="inlineStr">
+        <is>
+          <t>10-10-2026</t>
+        </is>
+      </c>
+      <c r="D18" s="25" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+      <c r="E18" s="25" t="inlineStr">
+        <is>
+          <t>Necesario</t>
+        </is>
+      </c>
+      <c r="F18" s="25" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="G18" s="24" t="inlineStr">
+        <is>
+          <t>Ampliar FS-HU-12 con el panel del administrador según el mockup del Product Owner (Dashboard, Profesionales, Verificaciones, Usuarios y Reportes; Configuración y Contenido quedan fuera), con solicitudes y documentos de verificación. Como Luis Méndez la implementó en el Sprint 3 (PR #15, #19 y #20), el 12-10-2026 se reubicó del Sprint 5 al Sprint 3 y el Product Owner la aceptó con una observación.</t>
+        </is>
+      </c>
+      <c r="H18" s="25" t="inlineStr">
+        <is>
+          <t>FS-HU-12</t>
+        </is>
+      </c>
+      <c r="I18" s="25" t="inlineStr">
+        <is>
+          <t>CU-07</t>
+        </is>
+      </c>
+      <c r="J18" s="24" t="inlineStr">
+        <is>
+          <t>Fase 2 – Sprint 3 (semanas 9 y 10)</t>
+        </is>
+      </c>
+      <c r="K18" s="25" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="L18" s="26" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="98" customHeight="1">
+      <c r="A19" s="23" t="inlineStr">
+        <is>
+          <t>SC-17</t>
+        </is>
+      </c>
+      <c r="B19" s="24" t="inlineStr">
+        <is>
+          <t>Rodrigo Cárcamo Rojas / Product Owner</t>
+        </is>
+      </c>
+      <c r="C19" s="25" t="inlineStr">
+        <is>
+          <t>12-10-2026</t>
+        </is>
+      </c>
+      <c r="D19" s="25" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+      <c r="E19" s="25" t="inlineStr">
+        <is>
+          <t>Necesario</t>
+        </is>
+      </c>
+      <c r="F19" s="25" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="G19" s="24" t="inlineStr">
+        <is>
+          <t>Limitar a una reserva activa (pendiente o confirmada) de un horario futuro por usuario con cada profesional; las citas que ya pasaron no cuentan. Si no se cumple, la API responde 409 con el motivo y la ficha avisa antes de escribir el mensaje. Se agregó el escenario 4 a FS-HU-14 y se implementó en el PR #22 (defecto 26 corregido).</t>
+        </is>
+      </c>
+      <c r="H19" s="25" t="inlineStr">
+        <is>
+          <t>FS-HU-14</t>
+        </is>
+      </c>
+      <c r="I19" s="25" t="inlineStr">
+        <is>
+          <t>CU-09</t>
+        </is>
+      </c>
+      <c r="J19" s="24" t="inlineStr">
+        <is>
+          <t>Fase 2 – Sprint 3 (semanas 9 y 10)</t>
+        </is>
+      </c>
+      <c r="K19" s="25" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="L19" s="26" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="15" customHeight="1"/>
+    <row r="21" ht="15" customHeight="1"/>
+    <row r="22" ht="15" customHeight="1">
+      <c r="A22" s="28" t="inlineStr">
         <is>
           <t>Notas:</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="28" customHeight="1">
-      <c r="A17" s="29" t="inlineStr">
+    <row r="23" ht="28" customHeight="1">
+      <c r="A23" s="29" t="inlineStr">
         <is>
           <t>• Solicitante: el cliente del proyecto está representado por el Product Owner; también se registran los cambios pedidos por el docente o propuestos por un integrante del equipo.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="28" customHeight="1">
-      <c r="A18" s="29" t="inlineStr">
+    <row r="24" ht="28" customHeight="1">
+      <c r="A24" s="29" t="inlineStr">
         <is>
           <t>• Requerimiento relacionado: FitSearch trabaja con Scrum y sus requerimientos funcionales son las historias de usuario del Product Backlog, por eso se indica el ID de la historia (FS-HU-N°). Los casos de uso (CU-N°) son los del Documento de Arquitectura del Sistema (DAS).</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="28" customHeight="1">
-      <c r="A19" s="29" t="inlineStr">
+    <row r="25" ht="28" customHeight="1">
+      <c r="A25" s="29" t="inlineStr">
         <is>
           <t>• El detalle y la justificación de cada cambio están en la sección 3 de la Guía 2.4, en el historial de versiones del DAS y en los comentarios del Product Backlog. Actualizado al 03-10-2026.</t>
         </is>
@@ -1557,11 +1917,11 @@
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A16:L16"/>
-    <mergeCell ref="A19:L19"/>
+    <mergeCell ref="A24:L24"/>
+    <mergeCell ref="A25:L25"/>
     <mergeCell ref="A1:L1"/>
-    <mergeCell ref="A17:L17"/>
-    <mergeCell ref="A18:L18"/>
+    <mergeCell ref="A23:L23"/>
+    <mergeCell ref="A22:L22"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1" horizontalDpi="4294967294" verticalDpi="0"/>

</xml_diff>

<commit_message>
SC-19: mejoras de interaccion de la interfaz y defectos 30 a 34
Scroll al cambiar de pantalla, confirmacion de la agenda en su tarjeta, busqueda sin saltos, campos de 16 px, boton principal en la agenda, respuesta al presionar, menus y paneles con transiciones y movimiento reducido. CP-081 a CP-087; Guia 2.4, control, matriz, planilla y registro de defectos al 19-10-2026.
</commit_message>
<xml_diff>
--- a/FASE 2/Evidencias Proyecto/Evidencias de documentación/Control del proyecto/Matriz_Control_de_Cambio_FitSearch.xlsx
+++ b/FASE 2/Evidencias Proyecto/Evidencias de documentación/Control del proyecto/Matriz_Control_de_Cambio_FitSearch.xlsx
@@ -737,7 +737,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L25"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1947,42 +1947,105 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1"/>
-    <row r="22" ht="15" customHeight="1">
-      <c r="A22" s="28" t="inlineStr">
+    <row r="21" ht="150" customHeight="1">
+      <c r="A21" s="23" t="inlineStr">
+        <is>
+          <t>SC-19</t>
+        </is>
+      </c>
+      <c r="B21" s="24" t="inlineStr">
+        <is>
+          <t>Rodrigo Cárcamo Rojas / Product Owner</t>
+        </is>
+      </c>
+      <c r="C21" s="25" t="inlineStr">
+        <is>
+          <t>19-10-2026</t>
+        </is>
+      </c>
+      <c r="D21" s="25" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+      <c r="E21" s="25" t="inlineStr">
+        <is>
+          <t>Necesario</t>
+        </is>
+      </c>
+      <c r="F21" s="25" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="G21" s="24" t="inlineStr">
+        <is>
+          <t>Mejorar la respuesta y el movimiento de la interfaz sin cambiar funciones: lo que se presiona se achica apenas; los efectos al pasar el mouse solo aplican con mouse; el menú lateral y la hoja de filtros del celular se abren con curva de cajón, con fondo que se funde y sin desplazar la página de fondo; los menús de la cuenta y de notificaciones crecen desde su botón; entradas breves en Elegir perfil y en el asistente de perfil; el corazón de favoritos late al marcarlo; se respeta la preferencia «reducir movimiento» y en el celular los campos usan 16 px y las pantallas 100dvh. Incluye la corrección de los defectos 30 a 34 (CP-081 a CP-087). Sin dependencias nuevas.</t>
+        </is>
+      </c>
+      <c r="H21" s="25" t="inlineStr">
+        <is>
+          <t>FS-HU-02, FS-HU-13, FS-HU-14, FS-HU-21 a FS-HU-23</t>
+        </is>
+      </c>
+      <c r="I21" s="25" t="inlineStr">
+        <is>
+          <t>CU-02, CU-03, CU-08, CU-09</t>
+        </is>
+      </c>
+      <c r="J21" s="24" t="inlineStr">
+        <is>
+          <t>Fase 2 – Sprint 4 (semanas 11 y 12)</t>
+        </is>
+      </c>
+      <c r="K21" s="25" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+      <c r="L21" s="26" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23" ht="15" customHeight="1">
+      <c r="A23" s="28" t="inlineStr">
         <is>
           <t>Notas:</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="28" customHeight="1">
-      <c r="A23" s="29" t="inlineStr">
-        <is>
-          <t>• Solicitante: el cliente del proyecto está representado por el Product Owner; también se registran los cambios pedidos por el docente o propuestos por un integrante del equipo.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="28" customHeight="1">
       <c r="A24" s="29" t="inlineStr">
         <is>
-          <t>• Requerimiento relacionado: FitSearch trabaja con Scrum y sus requerimientos funcionales son las historias de usuario del Product Backlog, por eso se indica el ID de la historia (FS-HU-N°). Los casos de uso (CU-N°) son los del Documento de Arquitectura del Sistema (DAS).</t>
+          <t>• Solicitante: el cliente del proyecto está representado por el Product Owner; también se registran los cambios pedidos por el docente o propuestos por un integrante del equipo.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="28" customHeight="1">
       <c r="A25" s="29" t="inlineStr">
         <is>
-          <t>• El detalle y la justificación de cada cambio están en la sección 3 de la Guía 2.4, en el historial de versiones del DAS y en los comentarios del Product Backlog. Actualizado al 03-10-2026.</t>
-        </is>
-      </c>
-    </row>
+          <t>• Requerimiento relacionado: FitSearch trabaja con Scrum y sus requerimientos funcionales son las historias de usuario del Product Backlog, por eso se indica el ID de la historia (FS-HU-N°). Los casos de uso (CU-N°) son los del Documento de Arquitectura del Sistema (DAS).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="28" customHeight="1">
+      <c r="A26" s="29" t="inlineStr">
+        <is>
+          <t>• El detalle y la justificación de cada cambio están en la sección 3 de la Guía 2.4, en el historial de versiones del DAS y en los comentarios del Product Backlog. Actualizado al 19-10-2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27"/>
   </sheetData>
   <mergeCells count="5">
+    <mergeCell ref="A26:L26"/>
     <mergeCell ref="A24:L24"/>
     <mergeCell ref="A25:L25"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A23:L23"/>
-    <mergeCell ref="A22:L22"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1" horizontalDpi="4294967294" verticalDpi="0"/>

</xml_diff>

<commit_message>
SC-28: ubicacion de la ficha profesional por direccion con Nominatim (DAS 1.28)
La ficha ya no pide latitud ni longitud: la API ubica la comuna y la direccion y el formulario muestra un mapa con marcador ajustable. CP-123 a CP-125, diagramas 07 y 08, Matriz, control, Product Backlog y README.
</commit_message>
<xml_diff>
--- a/FASE 2/Evidencias Proyecto/Evidencias de documentación/Control del proyecto/Matriz_Control_de_Cambio_FitSearch.xlsx
+++ b/FASE 2/Evidencias Proyecto/Evidencias de documentación/Control del proyecto/Matriz_Control_de_Cambio_FitSearch.xlsx
@@ -737,7 +737,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L35"/>
+  <dimension ref="A1:L36"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2505,43 +2505,105 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
-    <row r="31" ht="15" customHeight="1">
-      <c r="A31" s="28" t="inlineStr">
+    <row r="30" ht="225" customHeight="1">
+      <c r="A30" s="23" t="inlineStr">
+        <is>
+          <t>SC-28</t>
+        </is>
+      </c>
+      <c r="B30" s="24" t="inlineStr">
+        <is>
+          <t>Rodrigo Cárcamo Rojas / Product Owner</t>
+        </is>
+      </c>
+      <c r="C30" s="25" t="inlineStr">
+        <is>
+          <t>24-10-2026</t>
+        </is>
+      </c>
+      <c r="D30" s="25" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+      <c r="E30" s="25" t="inlineStr">
+        <is>
+          <t>Necesario</t>
+        </is>
+      </c>
+      <c r="F30" s="25" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="G30" s="24" t="inlineStr">
+        <is>
+          <t>Quitar los campos de latitud y longitud de la ficha del profesional, porque una persona común no sabe obtener coordenadas: el profesional escribe solo su comuna y su dirección, el backend las busca en Nominatim (el buscador de direcciones de OpenStreetMap, gratuito y sin clave) y el recuadro «Vista previa del mapa de ubicación» pasa a ser un mapa real con el marcador del lugar encontrado. Si no quedó exacto (por ejemplo, encontró la calle pero no el número), el profesional arrastra el marcador, hace clic en el mapa o lo mueve con las flechas del teclado. Nueva ruta GET /api/profesionales/mi-ficha/ubicacion (solo rol profesional), con una consulta por segundo, caché de 24 horas e identificación de la aplicación, como exige la política de uso de Nominatim. Sin cambios en la base de datos: la ficha sigue guardando latitud y longitud, y la API las sigue validando dentro de Chile. Retoma la alternativa que D32 había descartado (geocodificar la dirección). DAS 1.28 (D36) y diagramas 07 y 08 actualizados (CP-123 a CP-125).</t>
+        </is>
+      </c>
+      <c r="H30" s="25" t="inlineStr">
+        <is>
+          <t>FS-HU-04</t>
+        </is>
+      </c>
+      <c r="I30" s="25" t="inlineStr">
+        <is>
+          <t>CU-04</t>
+        </is>
+      </c>
+      <c r="J30" s="24" t="inlineStr">
+        <is>
+          <t>Fase 2 – Sprint 4 (semanas 11 y 12)</t>
+        </is>
+      </c>
+      <c r="K30" s="25" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="L30" s="26" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+    </row>
+    <row r="31"/>
+    <row r="32" ht="15" customHeight="1">
+      <c r="A32" s="28" t="inlineStr">
         <is>
           <t>Notas:</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="28" customHeight="1">
-      <c r="A32" s="29" t="inlineStr">
-        <is>
-          <t>• Solicitante: el cliente del proyecto está representado por el Product Owner; también se registran los cambios pedidos por el docente o propuestos por un integrante del equipo.</t>
         </is>
       </c>
     </row>
     <row r="33" ht="28" customHeight="1">
       <c r="A33" s="29" t="inlineStr">
         <is>
-          <t>• Requerimiento relacionado: FitSearch trabaja con Scrum y sus requerimientos funcionales son las historias de usuario del Product Backlog, por eso se indica el ID de la historia (FS-HU-N°). Los casos de uso (CU-N°) son los del Documento de Arquitectura del Sistema (DAS).</t>
+          <t>• Solicitante: el cliente del proyecto está representado por el Product Owner; también se registran los cambios pedidos por el docente o propuestos por un integrante del equipo.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="28" customHeight="1">
       <c r="A34" s="29" t="inlineStr">
         <is>
-          <t>• El detalle y la justificación de cada cambio están en la sección 3 de la Guía 2.4, en el historial de versiones del DAS y en los comentarios del Product Backlog. Actualizado al 19-10-2026.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35"/>
+          <t>• Requerimiento relacionado: FitSearch trabaja con Scrum y sus requerimientos funcionales son las historias de usuario del Product Backlog, por eso se indica el ID de la historia (FS-HU-N°). Los casos de uso (CU-N°) son los del Documento de Arquitectura del Sistema (DAS).</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="28" customHeight="1">
+      <c r="A35" s="29" t="inlineStr">
+        <is>
+          <t>• El detalle y la justificación de cada cambio están en la sección 3 de la Guía 2.4, en el historial de versiones del DAS y en los comentarios del Product Backlog. Actualizado al 24-10-2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36"/>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A33:L33"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A32:L32"/>
-    <mergeCell ref="A31:L31"/>
     <mergeCell ref="A34:L34"/>
+    <mergeCell ref="A35:L35"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1" horizontalDpi="4294967294" verticalDpi="0"/>

</xml_diff>